<commit_message>
Complete login page tests
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" state="visible" r:id="rId2"/>
@@ -259,6 +259,9 @@
 3. Password: InvPass</t>
   </si>
   <si>
+    <t xml:space="preserve">TC_0004</t>
+  </si>
+  <si>
     <t xml:space="preserve">Login using invalid username &amp; invalid password</t>
   </si>
   <si>
@@ -267,7 +270,7 @@
 3. Password: InvPass</t>
   </si>
   <si>
-    <t xml:space="preserve">TC_0004</t>
+    <t xml:space="preserve">TC_0005</t>
   </si>
   <si>
     <t xml:space="preserve">1. The browser is `MS Edge`
@@ -283,7 +286,7 @@
     <t xml:space="preserve">The main banner is visible</t>
   </si>
   <si>
-    <t xml:space="preserve">TC_0005</t>
+    <t xml:space="preserve">TC_0006</t>
   </si>
   <si>
     <t xml:space="preserve">Reset password with valid Username</t>
@@ -356,9 +359,6 @@
     <t xml:space="preserve">Quick Launch</t>
   </si>
   <si>
-    <t xml:space="preserve">TC_0006</t>
-  </si>
-  <si>
     <t xml:space="preserve">Buzz Latest Posts</t>
   </si>
   <si>
@@ -380,24 +380,8 @@
     <t xml:space="preserve">TC_0010</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SC_0007
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">SC_0008</t>
-    </r>
+    <t xml:space="preserve">SC_0007
+SC_0008</t>
   </si>
   <si>
     <t xml:space="preserve">Profile icon</t>
@@ -422,7 +406,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -450,11 +434,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -542,7 +521,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1196,7 +1175,7 @@
     </row>
     <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>23</v>
@@ -1205,13 +1184,13 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>63</v>
@@ -1228,7 +1207,7 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>26</v>
@@ -1240,19 +1219,19 @@
         <v>28</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>65</v>
@@ -1260,7 +1239,7 @@
     </row>
     <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>46</v>
@@ -1269,22 +1248,22 @@
         <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>65</v>
@@ -1329,7 +1308,7 @@
         <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1378,13 +1357,13 @@
         <v>32</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>63</v>
@@ -1407,25 +1386,25 @@
         <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>65</v>
@@ -1439,25 +1418,25 @@
         <v>37</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>65</v>
@@ -1465,31 +1444,31 @@
     </row>
     <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>65</v>
@@ -1497,31 +1476,31 @@
     </row>
     <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>65</v>
@@ -1529,7 +1508,7 @@
     </row>
     <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>37</v>
@@ -1538,22 +1517,22 @@
         <v>102</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>65</v>
@@ -1570,22 +1549,22 @@
         <v>104</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>65</v>
@@ -1599,25 +1578,25 @@
         <v>37</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>65</v>
@@ -1634,22 +1613,22 @@
         <v>107</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>65</v>
@@ -1669,10 +1648,10 @@
         <v>111</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>112</v>

</xml_diff>

<commit_message>
Complete test "Validate that, the profile item is visible on the page"
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Scenarios" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Login page" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard page" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Test Scenarios" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Login page" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Dashboard page" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Dashboard page'!$A$4:$K$4</definedName>
@@ -146,7 +146,7 @@
     <t xml:space="preserve">All dashboard widgets</t>
   </si>
   <si>
-    <t xml:space="preserve">Validate that, all widgets is displayed</t>
+    <t xml:space="preserve">Validate that, all widgets are displayed</t>
   </si>
   <si>
     <t xml:space="preserve">Medium</t>
@@ -543,13 +543,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFDDDDDD"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -629,13 +630,119 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.67"/>
@@ -1019,7 +1126,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:K10"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="12.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.35"/>
@@ -1288,7 +1395,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:K17"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="12.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.35"/>

</xml_diff>